<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.003-05 Raphaël et la porte fermée
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.003-05.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.003-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>rue de la bibliothèque puis maison</t>
+          <t>rue de la bibliothèque puis maison, store, façade, porte, sac, table, corbeille, fraises, pomme, livre</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raphaël, papa</t>
+          <t>Raphaël, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>La bibliothèque est fermée. Raphaël dit qu'il est déçu. Ils lisent à la maison. Plus tard, plus de fraises. Il choisit une pomme.</t>
+          <t>La barre de fer est froide. Sur les lamelles, un éclat de store luit. Raphaël veut entrer, maintenant. La porte est fermée. Sourire parti. Papa s'accroupit. Je suis déçu. Merci vécu. Ils lisent à la maison. Deuxième ruse : plus de fraises, la pomme glisse. Il refuse de foncer. Il choisit une pomme. Un éclat de store tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une flaque ronde brille sur le trottoir. Elle tient tout le ciel, tout petit. Le support à vélos goutte encore. Une goutte tombe, puis une autre. Un papier est collé sur la vitre. Les lettres sont un peu floues. La poignée de cuivre est froide. Tu as vu la flaque, Raphaël ? Elle est ronde. Comme un miroir. Tu as les mains froides ? Un peu. En ce moment, ils arrivent devant la porte. Raphaël pose la main sur la poignée. La porte ne s'ouvre pas. Elle est fermée, aujourd'hui. Raphaël sent ses épaules tomber. Sa gorge se serre. Je suis déçu. Tu es déçu. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Raphaël souffle une fois. Son souffle fait un petit nuage. On peut lire à la maison ? Une autre idée. Bravo, Raphaël. Ils rentrent. Le tapis de l'entrée est un peu mouillé. Raphaël enlève ses chaussures. Il choisit un livre de trains. Les pages sentent le papier. Tu veux que je lise ? Oui. Ils s'assoient sur le tapis. Le tapis est épais sous les genoux. Le train du livre a une cheminée rouge. Tu vois la petite roue ? Elle est noire. Plus tard, Raphaël a soif de fruit. Des fraises, papa ? Papa ouvre le bac. Le bac est vide, tout vide. Il n'y en a plus. Raphaël sent encore sa gorge. Je suis déçu. Encore un souhait qui attend. Une autre idée ? Raphaël regarde la corbeille. Une pomme, alors. Oui. Tu as proposé autre chose. Papa coupe la pomme. La chair est blanche et juteuse. Raphaël croque. C'est froid et sucré. Être déçu n'est pas honteux. Une autre idée peut venir. Le livre de trains reste ouvert sur les genoux.</t>
+          <t>La barre de fer est froide, près du trottoir. Elle pique, papa. Tu la touches, la barre ? Oui, papa. Maman pose un sac contre sa jambe. Il est lourd, maman. Tu le portes un peu, Raphaël ? Un peu, maman. Raphaël connaît la rue de la bibliothèque. C'est notre rue. Tu la reconnais, la rue ? Oui, papa. Un détail paraît nouveau, près de la façade. Le store est baissé. Tu le vois, le store ? Oui, maman. Les lamelles du store font un bruit sec. Ça claque un peu. Tu l'entends, le clac ? Oui. Sur les lamelles, un éclat de store luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Le sac froisse, près des genoux de maman. Il fait du bruit. Tu l'entends, le sac ? Oui. Le bouton du manteau tape le sac. Il fait toc. Tu l'entends, le toc ? Oui, papa. La porte de la bibliothèque attend, trop loin. On y va ! On avance, Raphaël ? Oui, papa. Les chaussures tapent le trottoir, trop vite. J'ai hâte. Tes pieds courent, Raphaël ? Un peu, maman. En ce moment, Raphaël tend la main vers la porte. Je veux entrer, maintenant ! Tout de suite ? Oui, papa. Raphaël pousse la porte, trop vite. La porte ne bouge pas. Elle est fermée. La bibliothèque, Raphaël ? Fermée. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Tu as les épaules lourdes, Raphaël ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Raphaël ? Un peu, maman. Je suis déçu. L'éclat de store tremble, puis tient. Tu vois la porte fermée ? Oui. Raphaël serre les poings, puis les ouvre. Tes poings, Raphaël ? Ils se desserrent.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une flaque ronde brille sur le trottoir. Elle tient tout le ciel, tout petit. Le support à vélos goutte encore. Une goutte tombe, puis une autre. Un papier est collé sur la vitre. Les lettres sont un peu floues. La poignée de cuivre est froide. Tu as vu la flaque, Raphaël ? Elle est ronde. Comme un miroir. Tu as les mains froides ? Un peu. En ce moment, ils arrivent devant la porte. Raphaël pose la main sur la poignée. La porte ne s'ouvre pas. Elle est fermée, aujourd'hui. Raphaël sent ses épaules tomber. Sa gorge se serre. Je suis déçu. Tu es déçu. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Raphaël souffle une fois. Son souffle fait un petit nuage. On peut lire à la maison ? Une autre idée. Bravo, Raphaël. Ils rentrent. Le tapis de l'entrée est un peu mouillé. Raphaël enlève ses chaussures. Il choisit un livre de trains. Les pages sentent le papier. Tu veux que je lise ? Oui. Ils s'assoient sur le tapis. Le tapis est épais sous les genoux. Le train du livre a une cheminée rouge. Tu vois la petite roue ? Elle est noire. Plus tard, Raphaël a soif de fruit. Des fraises, papa ? Papa ouvre le bac. Le bac est vide, tout vide. Il n'y en a plus. Raphaël sent encore sa gorge. Je suis déçu. Encore un souhait qui attend. Une autre idée ? Raphaël regarde la corbeille. Une pomme, alors. Oui. Tu as proposé autre chose. Papa coupe la pomme. La chair est blanche et juteuse. Raphaël croque. C'est froid et sucré. Être déçu n'est pas honteux. Une autre idée peut venir. Le livre de trains reste ouvert sur les genoux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La barre de fer est froide, près du trottoir. Elle pique, papa. Tu la touches, la barre ? Oui, papa. Maman pose un sac contre sa jambe. Il est lourd, maman. Tu le portes un peu, Raphaël ? Un peu, maman. Raphaël connaît la rue de la bibliothèque. C'est notre rue. Tu la reconnais, la rue ? Oui, papa. Un détail paraît nouveau, près de la façade. Le store est baissé. Tu le vois, le store ? Oui, maman. Les lamelles du store font un bruit sec. Ça claque un peu. Tu l'entends, le clac ? Oui. Sur les lamelles, un &lt;emphasis level="moderate"&gt;éclat de store&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Le sac froisse, près des genoux de maman. Il fait du bruit. Tu l'entends, le sac ? Oui. Le bouton du manteau tape le sac. Il fait toc. Tu l'entends, le toc ? Oui, papa. La porte de la bibliothèque attend, trop loin. On y va ! On avance, Raphaël ? Oui, papa. Les chaussures tapent le trottoir, trop vite. J'ai hâte. Tes pieds courent, Raphaël ? Un peu, maman. En ce moment, Raphaël tend la main vers la porte. Je veux entrer, maintenant ! Tout de suite ? Oui, papa. Raphaël pousse la porte, trop vite. La porte ne bouge pas. Elle est fermée. La bibliothèque, Raphaël ? Fermée. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Tu as les épaules lourdes, Raphaël ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Raphaël ? Un peu, maman. Je suis déçu. L'éclat de store tremble, puis tient. Tu vois la porte fermée ? Oui. Raphaël serre les poings, puis les ouvre. Tes poings, Raphaël ? Ils se desserrent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ugo veut aller à la bibliothèque avec papa. La porte est fermée. Ugo sent ses épaules tomber. Sa gorge se serre. Ugo dit : je suis &lt;emphasis&gt;déçu&lt;/emphasis&gt;. Papa s'accroupit. Papa dit : un souhait peut attendre. On peut chercher une autre idée. Ugo souffle. Il dit : on peut lire à la maison. Papa sourit. Ils rentrent. Ugo choisit un livre de trains. Plus tard, Ugo veut des fraises. Il n'y en a plus. Ugo sent encore sa gorge. Il dit : je suis déçu. Puis il cherche une autre idée. Il dit : une pomme, alors. Papa coupe la pomme. Être déçu n'est pas honteux. Une autre idée peut venir. [pause]</t>
+          <t>La barre de fer est froide, près du trottoir. Elle pique, papa. Tu la touches, la barre ? Oui, papa. Maman pose un sac contre sa jambe. Il est lourd, maman. Tu le portes un peu, Raphaël ? Un peu, maman. Raphaël connaît la rue de la bibliothèque. C'est notre rue. Tu la reconnais, la rue ? Oui, papa. Un détail paraît nouveau, près de la façade. Le store est baissé. Tu le vois, le store ? Oui, maman. Les lamelles du store font un bruit sec. Ça claque un peu. Tu l'entends, le clac ? Oui. Sur les lamelles, un &lt;emphasis&gt;éclat de store&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Le sac froisse, près des genoux de maman. Il fait du bruit. Tu l'entends, le sac ? Oui. Le bouton du manteau tape le sac. Il fait toc. Tu l'entends, le toc ? Oui, papa. La porte de la bibliothèque attend, trop loin. On y va ! On avance, Raphaël ? Oui, papa. Les chaussures tapent le trottoir, trop vite. J'ai hâte. Tes pieds courent, Raphaël ? Un peu, maman. En ce moment, Raphaël tend la main vers la porte. Je veux entrer, maintenant ! Tout de suite ? Oui, papa. Raphaël pousse la porte, trop vite. La porte ne bouge pas. Elle est fermée. La bibliothèque, Raphaël ? Fermée. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Tu as les épaules lourdes, Raphaël ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Raphaël ? Un peu, maman. Je suis déçu. L'éclat de store tremble, puis tient. Tu vois la porte fermée ? Oui. Raphaël serre les poings, puis les ouvre. Tes poings, Raphaël ? Ils se desserrent. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>éclat de store</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,69 +1321,83 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis déception; intensite=2; destinataire=enfant; sous_texte=il_veut_entrer_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une flaque ronde brille sur le trottoir.
-narrateur|Elle tient tout le ciel, tout petit.
-narrateur|Le support à vélos goutte encore.
-narrateur|Une goutte tombe, puis une autre.
-narrateur|Un papier est collé sur la vitre.
-narrateur|Les lettres sont un peu floues.
-narrateur|La poignée de cuivre est froide.
-papa|Tu as vu la flaque, Raphaël ?
-enfant-m|Elle est ronde.
-papa|Comme un miroir.
-papa|Tu as les mains froides ?
-enfant-m|Un peu.
-narrateur|En ce moment, ils arrivent devant la porte.
-narrateur|Raphaël pose la main sur la poignée.
-narrateur|La porte ne s'ouvre pas.
-papa|Elle est fermée, aujourd'hui.
-narrateur|Raphaël sent ses épaules tomber.
-narrateur|Sa gorge se serre.
+          <t>narrateur|La barre de fer est froide, près du trottoir.
+enfant-m|Elle pique, papa.
+papa|Tu la touches, la barre ?
+enfant-m|Oui, papa.
+narrateur|Maman pose un sac contre sa jambe.
+enfant-m|Il est lourd, maman.
+maman|Tu le portes un peu, Raphaël ?
+enfant-m|Un peu, maman.
+narrateur|Raphaël connaît la rue de la bibliothèque.
+enfant-m|C'est notre rue.
+papa|Tu la reconnais, la rue ?
+enfant-m|Oui, papa.
+narrateur|Un détail paraît nouveau, près de la façade.
+enfant-m|Le store est baissé.
+maman|Tu le vois, le store ?
+enfant-m|Oui, maman.
+narrateur|Les lamelles du store font un bruit sec.
+enfant-m|Ça claque un peu.
+papa|Tu l'entends, le clac ?
+enfant-m|Oui.
+narrateur|Sur les lamelles, un éclat de store luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-m|Oui, un point clair.
+narrateur|Le sac froisse, près des genoux de maman.
+enfant-m|Il fait du bruit.
+maman|Tu l'entends, le sac ?
+enfant-m|Oui.
+narrateur|Le bouton du manteau tape le sac.
+enfant-m|Il fait toc.
+papa|Tu l'entends, le toc ?
+enfant-m|Oui, papa.
+narrateur|La porte de la bibliothèque attend, trop loin.
+enfant-m|On y va !
+papa|On avance, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Les chaussures tapent le trottoir, trop vite.
+enfant-m|J'ai hâte.
+maman|Tes pieds courent, Raphaël ?
+enfant-m|Un peu, maman.
+narrateur|En ce moment, Raphaël tend la main vers la porte.
+enfant-m|Je veux entrer, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Raphaël pousse la porte, trop vite.
+narrateur|La porte ne bouge pas.
+enfant-m|Elle est fermée.
+maman|La bibliothèque, Raphaël ?
+enfant-m|Fermée.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+enfant-m|J'ai mal au ventre.
+papa|Tu as les épaules lourdes, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+maman|Tes mains sont chaudes, Raphaël ?
+enfant-m|Un peu, maman.
 enfant-m|Je suis déçu.
-papa|Tu es déçu.
-papa|Ce n'est pas honteux.
-papa|Un souhait peut attendre.
-papa|On peut chercher une autre idée.
-narrateur|Raphaël souffle une fois.
-narrateur|Son souffle fait un petit nuage.
-enfant-m|On peut lire à la maison ?
-papa|Une autre idée.
-papa|Bravo, Raphaël.
-narrateur|Ils rentrent.
-narrateur|Le tapis de l'entrée est un peu mouillé.
-narrateur|Raphaël enlève ses chaussures.
-narrateur|Il choisit un livre de trains.
-narrateur|Les pages sentent le papier.
-papa|Tu veux que je lise ?
+narrateur|L'éclat de store tremble, puis tient.
+papa|Tu vois la porte fermée ?
 enfant-m|Oui.
-narrateur|Ils s'assoient sur le tapis.
-narrateur|Le tapis est épais sous les genoux.
-narrateur|Le train du livre a une cheminée rouge.
-papa|Tu vois la petite roue ?
-enfant-m|Elle est noire.
-narrateur|Plus tard, Raphaël a soif de fruit.
-enfant-m|Des fraises, papa ?
-narrateur|Papa ouvre le bac.
-narrateur|Le bac est vide, tout vide.
-papa|Il n'y en a plus.
-narrateur|Raphaël sent encore sa gorge.
-enfant-m|Je suis déçu.
-papa|Encore un souhait qui attend.
-papa|Une autre idée ?
-narrateur|Raphaël regarde la corbeille.
-enfant-m|Une pomme, alors.
-papa|Oui.
-papa|Tu as proposé autre chose.
-narrateur|Papa coupe la pomme.
-narrateur|La chair est blanche et juteuse.
-narrateur|Raphaël croque.
-enfant-m|C'est froid et sucré.
-papa|Être déçu n'est pas honteux.
-papa|Une autre idée peut venir.
-narrateur|Le livre de trains reste ouvert sur les genoux.</t>
+narrateur|Raphaël serre les poings, puis les ouvre.
+papa|Tes poings, Raphaël ?
+enfant-m|Ils se desserrent.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>rue,store</t>
         </is>
       </c>
     </row>
@@ -1415,12 +1429,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>La bibliothèque est fermée. Que dit Raphaël ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La bibliothèque est fermée. Que dit &lt;emphasis level="moderate"&gt;Raphaël&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>La bibliothèque est fermée. Que dit Ugo ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;La bibliothèque est fermée. Que dit &lt;emphasis&gt;Raphaël&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1445,7 +1459,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Ugo cherche une autre idée. Que dit-il d'abord ?</t>
+          <t>Raphaël cherche une autre idée. Que dit-il d'abord ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1483,18 +1497,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1509,34 +1523,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Raphaël</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1545,23 +1563,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=la_bibliotheque_est_fermee_que_dit_raphael; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1594,17 +1612,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a encore un morceau de pomme. J'ai dit : je suis déçu. Oui. Le souhait peut attendre. Une autre idée est arrivée. Le livre, puis la pomme. Bravo, Raphaël. Deux autres idées. Oui. Le jus de pomme brille sur sa lèvre.</t>
+          <t>Raphaël avance la main vers la porte, trop vite. J'ouvre, maintenant ! Les mots se bousculent dans sa bouche. N'importe quoi. Raphaël avance les mains, trop vite. Puis il s'arrête. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le store, un instant. Il écoute la rue, près de la façade. À la maison, alors. Tu lis à la maison ? Oui, un livre. Merci, Raphaël. Papa reste à la même hauteur. Le sac est froid, sous les doigts. Il pique un peu. Ils marchent vers la maison, sans se presser. Raphaël tient le sac, tout petit. Il est lourd. Tu le portes, Raphaël ? Oui, papa. Tes pieds sont lents, Raphaël ? Oui, maman. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On rentre, après la rue ? Oui. Raphaël reprend le sac, sans se bousculer. Il vient avec nous. Tes mains sont au chaud, Raphaël ? Un peu, maman. La maison, plus tard. Oui, papa. Le sac reste contre sa chemise. Il est un peu froid.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a encore un morceau de pomme. J'ai dit : je suis déçu. Oui. Le souhait peut attendre. Une autre idée est arrivée. Le livre, puis la pomme. Bravo, Raphaël. Deux autres idées. Oui. Le jus de pomme brille sur sa lèvre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël avance la main vers la porte, trop vite. J'ouvre, maintenant ! Les mots se bousculent dans sa bouche. N'importe quoi. Raphaël avance les mains, trop vite. Puis il s'arrête. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le store, un instant. Il écoute la rue, près de la façade. À la maison, alors. Tu lis à la maison ? Oui, un &lt;emphasis level="moderate"&gt;livre&lt;/emphasis&gt;. Merci, Raphaël. Papa reste à la même hauteur. Le sac est froid, sous les doigts. Il pique un peu. Ils marchent vers la maison, sans se presser. Raphaël tient le sac, tout petit. Il est lourd. Tu le portes, Raphaël ? Oui, papa. Tes pieds sont lents, Raphaël ? Oui, maman. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On rentre, après la rue ? Oui. Raphaël reprend le sac, sans se bousculer. Il vient avec nous. Tes mains sont au chaud, Raphaël ? Un peu, maman. La maison, plus tard. Oui, papa. Le sac reste contre sa chemise. Il est un peu froid.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ugo a nommé : &lt;emphasis&gt;déçu&lt;/emphasis&gt;. Le souhait peut attendre. Une autre idée est arrivée. Papa était là. [pause]</t>
+          <t>Raphaël avance la main vers la porte, trop vite. J'ouvre, maintenant ! Les mots se bousculent dans sa bouche. N'importe quoi. Raphaël avance les mains, trop vite. Puis il s'arrête. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le store, un instant. Il écoute la rue, près de la façade. À la maison, alors. Tu lis à la maison ? Oui, un &lt;emphasis&gt;livre&lt;/emphasis&gt;. Merci, Raphaël. Papa reste à la même hauteur. Le sac est froid, sous les doigts. Il pique un peu. Ils marchent vers la maison, sans se presser. Raphaël tient le sac, tout petit. Il est lourd. Tu le portes, Raphaël ? Oui, papa. Tes pieds sont lents, Raphaël ? Oui, maman. Le ventre de Raphaël se desserre. Les épaules se relèvent un peu. On rentre, après la rue ? Oui. Raphaël reprend le sac, sans se bousculer. Il vient avec nous. Tes mains sont au chaud, Raphaël ? Un peu, maman. La maison, plus tard. Oui, papa. Le sac reste contre sa chemise. Il est un peu froid. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1651,7 +1669,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1659,10 +1677,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1685,30 +1703,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>livre</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1717,10 +1735,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1733,21 +1751,48 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_propose_de_lire_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël a encore un morceau de pomme.
-enfant-m|J'ai dit : je suis déçu.
-papa|Oui.
-papa|Le souhait peut attendre.
-papa|Une autre idée est arrivée.
-papa|Le livre, puis la pomme.
-papa|Bravo, Raphaël.
-enfant-m|Deux autres idées.
-papa|Oui.
-narrateur|Le jus de pomme brille sur sa lèvre.</t>
+          <t>narrateur|Raphaël avance la main vers la porte, trop vite.
+enfant-m|J'ouvre, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|N'importe quoi.
+narrateur|Raphaël avance les mains, trop vite.
+narrateur|Puis il s'arrête.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le store, un instant.
+narrateur|Il écoute la rue, près de la façade.
+enfant-m|À la maison, alors.
+papa|Tu lis à la maison ?
+enfant-m|Oui, un livre.
+papa|Merci, Raphaël.
+narrateur|Papa reste à la même hauteur.
+maman|Le sac est froid, sous les doigts.
+enfant-m|Il pique un peu.
+narrateur|Ils marchent vers la maison, sans se presser.
+narrateur|Raphaël tient le sac, tout petit.
+enfant-m|Il est lourd.
+papa|Tu le portes, Raphaël ?
+enfant-m|Oui, papa.
+maman|Tes pieds sont lents, Raphaël ?
+enfant-m|Oui, maman.
+narrateur|Le ventre de Raphaël se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On rentre, après la rue ?
+enfant-m|Oui.
+narrateur|Raphaël reprend le sac, sans se bousculer.
+enfant-m|Il vient avec nous.
+maman|Tes mains sont au chaud, Raphaël ?
+enfant-m|Un peu, maman.
+papa|La maison, plus tard.
+enfant-m|Oui, papa.
+narrateur|Le sac reste contre sa chemise.
+enfant-m|Il est un peu froid.</t>
         </is>
       </c>
     </row>
@@ -1774,17 +1819,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël croque encore la pomme. Papa range le marque-page. On s'assoit un peu ? Oui, papa. Tu as nommé : déçu. Puis tu as cherché. Le livre de trains reste ouvert. Une goutte sèche encore sur le rebord. Le train a une cheminée rouge. On le regardera encore.</t>
+          <t>La maison sent le bois, près de la table. Ça sent le bois, maman. Tu le sens, le bois ? Oui. Un livre de trains attend sur la table. Des fraises, maintenant ! Raphaël ouvre la corbeille, trop vite. La corbeille tremble, presque vide. Il n'y en a plus. Les fraises, Raphaël ? Parti. Les épaules de Raphaël retombent. Je les prends, tout de suite ! Raphaël avance trop vite vers la corbeille. Une pomme glisse au bord. Elle part ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la corbeille, un instant. Il écoute la maison, près du store. Sur le store, un éclat de store luit. Là, sur le store. On tient la pomme ? Oui, papa. La peau de la pomme résiste, un moment. Une pomme, alors. Tu la vois, la pomme ? Oui, maman. Papa coupe la pomme, sans se presser. La pomme cède, tout petit. Elle s'ouvre ! Ils lisent le livre, ensemble. Le train est prêt, Raphaël ? Oui, papa. Le jus de pomme colle un peu au doigt. Ça tient.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël croque encore la pomme. Papa range le marque-page. On s'assoit un peu ? Oui, papa. Tu as nommé : déçu. Puis tu as cherché. Le livre de trains reste ouvert. Une goutte sèche encore sur le rebord. Le train a une cheminée rouge. On le regardera encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La maison sent le bois, près de la table. Ça sent le bois, maman. Tu le sens, le bois ? Oui. Un livre de trains attend sur la table. Des fraises, maintenant ! Raphaël ouvre la corbeille, trop vite. La corbeille tremble, presque vide. Il n'y en a plus. Les fraises, Raphaël ? Parti. Les épaules de Raphaël retombent. Je les prends, tout de suite ! Raphaël avance trop vite vers la corbeille. Une pomme glisse au bord. Elle part ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la corbeille, un instant. Il écoute la maison, près du store. Sur le store, un &lt;emphasis level="moderate"&gt;éclat de store&lt;/emphasis&gt; luit. Là, sur le store. On tient la pomme ? Oui, papa. La peau de la pomme résiste, un moment. Une pomme, alors. Tu la vois, la pomme ? Oui, maman. Papa coupe la pomme, sans se presser. La pomme cède, tout petit. Elle s'ouvre ! Ils lisent le livre, ensemble. Le train est prêt, Raphaël ? Oui, papa. Le jus de pomme colle un peu au doigt. Ça tient.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ugo croque la pomme. Papa range le livre. Ils s'assoient. [pause]</t>
+          <t>La maison sent le bois, près de la table. Ça sent le bois, maman. Tu le sens, le bois ? Oui. Un livre de trains attend sur la table. Des fraises, maintenant ! Raphaël ouvre la corbeille, trop vite. La corbeille tremble, presque vide. Il n'y en a plus. Les fraises, Raphaël ? Parti. Les épaules de Raphaël retombent. Je les prends, tout de suite ! Raphaël avance trop vite vers la corbeille. Une pomme glisse au bord. Elle part ! Raphaël avance les mains, trop vite. Puis il s'arrête net. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la corbeille, un instant. Il écoute la maison, près du store. Sur le store, un &lt;emphasis&gt;éclat de store&lt;/emphasis&gt; luit. Là, sur le store. On tient la pomme ? Oui, papa. La peau de la pomme résiste, un moment. Une pomme, alors. Tu la vois, la pomme ? Oui, maman. Papa coupe la pomme, sans se presser. La pomme cède, tout petit. Elle s'ouvre ! Ils lisent le livre, ensemble. Le train est prêt, Raphaël ? Oui, papa. Le jus de pomme colle un peu au doigt. Ça tient. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1831,7 +1876,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1839,10 +1884,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1863,28 +1908,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de store</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1893,10 +1942,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1907,19 +1956,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=plus_de_fraises_il_refuse_de_foncer_il_choisit_une_pomme; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël croque encore la pomme.
-narrateur|Papa range le marque-page.
-papa|On s'assoit un peu ?
+          <t>narrateur|La maison sent le bois, près de la table.
+enfant-m|Ça sent le bois, maman.
+maman|Tu le sens, le bois ?
+enfant-m|Oui.
+narrateur|Un livre de trains attend sur la table.
+enfant-m|Des fraises, maintenant !
+narrateur|Raphaël ouvre la corbeille, trop vite.
+narrateur|La corbeille tremble, presque vide.
+enfant-m|Il n'y en a plus.
+maman|Les fraises, Raphaël ?
+enfant-m|Parti.
+narrateur|Les épaules de Raphaël retombent.
+enfant-m|Je les prends, tout de suite !
+narrateur|Raphaël avance trop vite vers la corbeille.
+narrateur|Une pomme glisse au bord.
+enfant-m|Elle part !
+narrateur|Raphaël avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Raphaël refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la corbeille, un instant.
+narrateur|Il écoute la maison, près du store.
+narrateur|Sur le store, un éclat de store luit.
+enfant-m|Là, sur le store.
+papa|On tient la pomme ?
 enfant-m|Oui, papa.
-papa|Tu as nommé : déçu.
-papa|Puis tu as cherché.
-narrateur|Le livre de trains reste ouvert.
-narrateur|Une goutte sèche encore sur le rebord.
-enfant-m|Le train a une cheminée rouge.
-papa|On le regardera encore.</t>
+narrateur|La peau de la pomme résiste, un moment.
+enfant-m|Une pomme, alors.
+maman|Tu la vois, la pomme ?
+enfant-m|Oui, maman.
+narrateur|Papa coupe la pomme, sans se presser.
+narrateur|La pomme cède, tout petit.
+enfant-m|Elle s'ouvre !
+narrateur|Ils lisent le livre, ensemble.
+papa|Le train est prêt, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Le jus de pomme colle un peu au doigt.
+enfant-m|Ça tient.</t>
         </is>
       </c>
     </row>
@@ -1946,17 +2028,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçu. J'ai trouvé une autre idée. Bravo, Raphaël. La pomme est finie, presque.</t>
+          <t>Ils restent près de la table. Maman essuie un peu de jus. La porte n'était pas ouverte, papa. Tu l'as vue, toi ? Oui, la porte fermée. On est bien, ici. Raphaël tapote le livre du doigt. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La pomme est restée, Raphaël. Oui, avec le livre. Ça sent le bois, un peu tiède. Et le store, maman. Oui, dans l'air. La maison est tiède, Raphaël ? Oui, papa. Le livre reste près de la pomme. Un éclat de store tient sur le tissu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçu. J'ai trouvé une autre idée. Bravo, Raphaël. La pomme est finie, presque.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Maman essuie un peu de jus. La porte n'était pas ouverte, papa. Tu l'as vue, toi ? Oui, la porte fermée. On est bien, ici. Raphaël tapote le livre du doigt. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La pomme est restée, Raphaël. Oui, avec le livre. Ça sent le bois, un peu tiède. Et le store, maman. Oui, dans l'air. La maison est tiède, Raphaël ? Oui, papa. Le livre reste près de la pomme. Un &lt;emphasis level="moderate"&gt;éclat de store&lt;/emphasis&gt; tient sur le tissu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Maman essuie un peu de jus. La porte n'était pas ouverte, papa. Tu l'as vue, toi ? Oui, la porte fermée. On est bien, ici. Raphaël tapote le livre du doigt. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La pomme est restée, Raphaël. Oui, avec le livre. Ça sent le bois, un peu tiède. Et le store, maman. Oui, dans l'air. La maison est tiède, Raphaël ? Oui, papa. Le livre reste près de la pomme. Un &lt;emphasis&gt;éclat de store&lt;/emphasis&gt; tient sur le tissu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2003,18 +2085,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2023,12 +2105,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2037,17 +2119,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de store</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2056,11 +2142,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2069,27 +2155,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_tissu; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit : je suis déçu.
-enfant-m|J'ai trouvé une autre idée.
-papa|Bravo, Raphaël.
-narrateur|La pomme est finie, presque.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Maman essuie un peu de jus.
+enfant-m|La porte n'était pas ouverte, papa.
+papa|Tu l'as vue, toi ?
+enfant-m|Oui, la porte fermée.
+maman|On est bien, ici.
+narrateur|Raphaël tapote le livre du doigt.
+enfant-m|Il a une trace de jus.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|La pomme est restée, Raphaël.
+enfant-m|Oui, avec le livre.
+narrateur|Ça sent le bois, un peu tiède.
+enfant-m|Et le store, maman.
+maman|Oui, dans l'air.
+papa|La maison est tiède, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Le livre reste près de la pomme.
+narrateur|Un éclat de store tient sur le tissu.</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2160,6 +2265,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>